<commit_message>
fix(P1): remove remaining devaluing copy in 395 calculator
</commit_message>
<xml_diff>
--- a/tools/candidates/p1-395-content-20261012/14-raschet-procentov-395-gk.xlsx
+++ b/tools/candidates/p1-395-content-20261012/14-raschet-procentov-395-gk.xlsx
@@ -773,7 +773,7 @@
     <row r="47" ht="98" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>В этой таблице учитывайте только сумму оплаты, направленную на погашение основного долга. По ст. 319 ГК РФ при недостаточности платежа сначала погашаются издержки кредитора по получению исполнения и проценты, являющиеся платой за пользование денежными средствами, затем основной долг. Проценты за просрочку по ст. 395 ГК РФ погашаются после основного долга (п. 49 постановления Пленума ВС РФ от 24.03.2016 № 7). Соглашением сторон можно изменить очередность только требований, названных в ст. 319 ГК РФ (п. 37 постановления Пленума ВС РФ от 22.11.2016 № 54). Если платёж распределяется между несколькими обязательствами или включает иные требования, уточните сумму погашения основного долга с юристом. База долга уменьшается со дня, следующего за датой оплаты; в день оплаты проценты начисляются на прежнюю сумму.</t>
+          <t>В этой таблице учитывайте только сумму оплаты, направленную на погашение основного долга. По ст. 319 ГК РФ при недостаточности платежа сначала погашаются издержки кредитора по получению исполнения и проценты, являющиеся платой за пользование денежными средствами, затем основной долг. Проценты за просрочку по ст. 395 ГК РФ погашаются после основного долга (п. 49 постановления Пленума ВС РФ от 24.03.2016 № 7). Соглашением сторон можно изменить очередность только требований, названных в ст. 319 ГК РФ (п. 37 постановления Пленума ВС РФ от 22.11.2016 № 54). Если платёж распределяется между несколькими обязательствами или включает иные требования, выделите сумму погашения основного долга по документам расчётов. База долга уменьшается со дня, следующего за датой оплаты; в день оплаты проценты начисляются на прежнюю сумму.</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
     <row r="48" ht="46" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Число дней в году берётся фактическое — 365 или 366. Формула считает по фактическому числу дней; норму, которая устанавливала бы иной знаменатель, этот расчёт не применяет. Если для вашего спора знаменатель принципиален, сверьте его с юристом по действующей практике на дату расчёта.</t>
+          <t>Число дней в году берётся фактическое — 365 или 366. Формула считает по фактическому числу дней; норму, которая устанавливала бы иной знаменатель, этот расчёт не применяет. Если порядок расчёта требует иного знаменателя, зафиксируйте его основание и применимость на дату расчёта.</t>
         </is>
       </c>
     </row>
@@ -2172,35 +2172,35 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Что это не заменяет</t>
+          <t>Условия применения расчёта</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>— Выбор между процентами по ст. 395 и договорной неустойкой. Если договором установлена неустойка за просрочку оплаты, по общему правилу взыскивается она (п. 4 ст. 395 ГК РФ) — выбор согласуйте с юристом.</t>
+          <t>— Сопоставьте условия договора об ответственности за просрочку оплаты с п. 4 ст. 395 ГК РФ. Если предусмотрена договорная неустойка, по общему правилу применяется она, если иное не установлено законом или договором.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>— Учёт мораторных периодов, банкротства должника и иных оснований приостановки начисления. При таких обстоятельствах расчёт корректирует юрист.</t>
+          <t>— Проверьте наличие мораториев, процедур банкротства и иных оснований ограничения начисления; при необходимости скорректируйте расчётный период и исходные данные.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>— Заключение специалиста. Суд проверяет расчёт сам; эта таблица — рабочий инструмент истца, а не доказательство само по себе.</t>
+          <t>— Подготовьте расчёт и подтверждающие документы: договор, акты, сведения об оплате, период просрочки и применённые ставки.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>— Сверку применимых условий договора, фактических обстоятельств и нормативных оснований начисления процентов.</t>
+          <t>— Сверьте применимые условия договора, фактические обстоятельства и нормативные основания начисления процентов.</t>
         </is>
       </c>
     </row>

</xml_diff>